<commit_message>
fix: dong bo ban ve va bang thong ke dinh kem tren web voi mat bang neo da ra soat (32 de dung chung, 92,2 m3)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/docs_huoi_vanh/HOHUOIVANH_BANG_THONG_KE_NEO_9_BE_PA3_DE_VIT.xlsx
+++ b/public/docs_huoi_vanh/HOHUOIVANH_BANG_THONG_KE_NEO_9_BE_PA3_DE_VIT.xlsx
@@ -3184,13 +3184,13 @@
         <v>BÈ 3</v>
       </c>
       <c r="D49">
-        <v>-41.3</v>
+        <v>-35.8</v>
       </c>
       <c r="E49">
-        <v>-149.57</v>
+        <v>-179.26</v>
       </c>
       <c r="F49">
-        <v>384.08</v>
+        <v>385.08</v>
       </c>
       <c r="G49">
         <v>1</v>
@@ -7462,13 +7462,13 @@
         <v>BÈ 5A</v>
       </c>
       <c r="D118">
-        <v>419.48</v>
+        <v>423.01</v>
       </c>
       <c r="E118">
-        <v>-154.12</v>
+        <v>-168.16</v>
       </c>
       <c r="F118">
-        <v>384.2</v>
+        <v>388.57</v>
       </c>
       <c r="G118">
         <v>1</v>
@@ -7524,13 +7524,13 @@
         <v>BÈ 5A</v>
       </c>
       <c r="D119">
-        <v>420.28</v>
+        <v>418.19</v>
       </c>
       <c r="E119">
-        <v>-149.28</v>
+        <v>-162.96</v>
       </c>
       <c r="F119">
-        <v>384.75</v>
+        <v>384</v>
       </c>
       <c r="G119">
         <v>1</v>
@@ -10748,13 +10748,13 @@
         <v>BÈ 7</v>
       </c>
       <c r="D171">
-        <v>76.46</v>
+        <v>81.73</v>
       </c>
       <c r="E171">
-        <v>-76.01</v>
+        <v>-97.29</v>
       </c>
       <c r="F171">
-        <v>384.07</v>
+        <v>384.1</v>
       </c>
       <c r="G171">
         <v>1</v>
@@ -12484,13 +12484,13 @@
         <v>BÈ 8</v>
       </c>
       <c r="D199">
-        <v>41.03</v>
+        <v>47.33</v>
       </c>
       <c r="E199">
-        <v>92.56</v>
+        <v>71.85</v>
       </c>
       <c r="F199">
-        <v>384.03</v>
+        <v>384.01</v>
       </c>
       <c r="G199">
         <v>1</v>
@@ -15048,19 +15048,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E7">
-        <v>-139.37</v>
+        <v>-138.58</v>
       </c>
       <c r="F7">
-        <v>30.03</v>
+        <v>31.21</v>
       </c>
       <c r="G7">
         <v>378.3</v>
       </c>
       <c r="H7">
-        <v>11.07</v>
+        <v>11.3</v>
       </c>
       <c r="I7">
-        <v>143.4</v>
+        <v>136.6</v>
       </c>
       <c r="J7">
         <v>2.5</v>
@@ -15090,10 +15090,10 @@
         <v>0.47</v>
       </c>
       <c r="S7">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="T7">
-        <v>0.5</v>
+        <v>0.47</v>
       </c>
       <c r="U7">
         <v>0</v>
@@ -15196,19 +15196,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E9">
-        <v>-48.11</v>
+        <v>-48.54</v>
       </c>
       <c r="F9">
-        <v>-33.37</v>
+        <v>-35.03</v>
       </c>
       <c r="G9">
         <v>378.3</v>
       </c>
       <c r="H9">
-        <v>8.91</v>
+        <v>9.01</v>
       </c>
       <c r="I9">
-        <v>102.6</v>
+        <v>113.6</v>
       </c>
       <c r="J9">
         <v>2.5</v>
@@ -15235,16 +15235,16 @@
         <v>38.6</v>
       </c>
       <c r="R9">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="S9">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="T9">
-        <v>0.69</v>
+        <v>0.67</v>
       </c>
       <c r="U9">
-        <v>0.43</v>
+        <v>0.38</v>
       </c>
       <c r="V9">
         <v>0.15</v>
@@ -15270,19 +15270,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E10">
-        <v>-25.86</v>
+        <v>-28.46</v>
       </c>
       <c r="F10">
-        <v>-15.46</v>
+        <v>-18.93</v>
       </c>
       <c r="G10">
         <v>378.3</v>
       </c>
       <c r="H10">
-        <v>13.98</v>
+        <v>14.23</v>
       </c>
       <c r="I10">
-        <v>121.3</v>
+        <v>138.9</v>
       </c>
       <c r="J10">
         <v>2.5</v>
@@ -15309,16 +15309,16 @@
         <v>38.6</v>
       </c>
       <c r="R10">
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="S10">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="T10">
-        <v>0.56</v>
+        <v>0.51</v>
       </c>
       <c r="U10">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
       <c r="V10">
         <v>0.15</v>
@@ -15344,19 +15344,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E11">
-        <v>18.01</v>
+        <v>16.6</v>
       </c>
       <c r="F11">
-        <v>-122.77</v>
+        <v>-124.06</v>
       </c>
       <c r="G11">
         <v>378.3</v>
       </c>
       <c r="H11">
-        <v>9.54</v>
+        <v>9.35</v>
       </c>
       <c r="I11">
-        <v>126.5</v>
+        <v>138</v>
       </c>
       <c r="J11">
         <v>3.25</v>
@@ -15383,16 +15383,16 @@
         <v>73.7</v>
       </c>
       <c r="R11">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="S11">
-        <v>0.62</v>
+        <v>0.55</v>
       </c>
       <c r="T11">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="U11">
-        <v>0.71</v>
+        <v>0.68</v>
       </c>
       <c r="V11">
         <v>0.15</v>
@@ -15418,34 +15418,34 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E12">
-        <v>49.15</v>
+        <v>42.39</v>
       </c>
       <c r="F12">
-        <v>-116.18</v>
+        <v>-119.37</v>
       </c>
       <c r="G12">
         <v>378.3</v>
       </c>
       <c r="H12">
-        <v>15.18</v>
+        <v>15.33</v>
       </c>
       <c r="I12">
-        <v>116.8</v>
+        <v>139.5</v>
       </c>
       <c r="J12">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="K12">
         <v>0.4</v>
       </c>
       <c r="L12">
-        <v>3.01</v>
+        <v>2.48</v>
       </c>
       <c r="M12">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="N12">
-        <v>7.7</v>
+        <v>6.4</v>
       </c>
       <c r="O12">
         <v>4</v>
@@ -15457,16 +15457,16 @@
         <v>73.7</v>
       </c>
       <c r="R12">
-        <v>0.62</v>
+        <v>0.73</v>
       </c>
       <c r="S12">
-        <v>0.69</v>
+        <v>0.75</v>
       </c>
       <c r="T12">
         <v>0.91</v>
       </c>
       <c r="U12">
-        <v>0.84</v>
+        <v>0.93</v>
       </c>
       <c r="V12">
         <v>0.15</v>
@@ -15492,34 +15492,34 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E13">
-        <v>33.69</v>
+        <v>29.5</v>
       </c>
       <c r="F13">
-        <v>-119.71</v>
+        <v>-121.71</v>
       </c>
       <c r="G13">
         <v>378.3</v>
       </c>
       <c r="H13">
-        <v>11.97</v>
+        <v>12.34</v>
       </c>
       <c r="I13">
-        <v>120.7</v>
+        <v>138.9</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="K13">
         <v>0.4</v>
       </c>
       <c r="L13">
-        <v>3.58</v>
+        <v>3.01</v>
       </c>
       <c r="M13">
-        <v>165</v>
+        <v>141</v>
       </c>
       <c r="N13">
-        <v>9.2</v>
+        <v>7.7</v>
       </c>
       <c r="O13">
         <v>4</v>
@@ -15531,16 +15531,16 @@
         <v>73.7</v>
       </c>
       <c r="R13">
-        <v>0.69</v>
+        <v>0.78</v>
       </c>
       <c r="S13">
-        <v>0.83</v>
+        <v>0.67</v>
       </c>
       <c r="T13">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="U13">
-        <v>0.74</v>
+        <v>0.92</v>
       </c>
       <c r="V13">
         <v>0.15</v>
@@ -15566,34 +15566,34 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E14">
-        <v>0.59</v>
+        <v>5.97</v>
       </c>
       <c r="F14">
-        <v>-131.46</v>
+        <v>-128.68</v>
       </c>
       <c r="G14">
         <v>378.3</v>
       </c>
       <c r="H14">
-        <v>9.76</v>
+        <v>9.59</v>
       </c>
       <c r="I14">
-        <v>172.3</v>
+        <v>135.9</v>
       </c>
       <c r="J14">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="K14">
         <v>0.4</v>
       </c>
       <c r="L14">
-        <v>4.21</v>
+        <v>3.58</v>
       </c>
       <c r="M14">
-        <v>202</v>
+        <v>165</v>
       </c>
       <c r="N14">
-        <v>10.8</v>
+        <v>9.2</v>
       </c>
       <c r="O14">
         <v>4</v>
@@ -15605,16 +15605,16 @@
         <v>73.7</v>
       </c>
       <c r="R14">
-        <v>0.66</v>
+        <v>0.84</v>
       </c>
       <c r="S14">
-        <v>0.58</v>
+        <v>0.61</v>
       </c>
       <c r="T14">
-        <v>0.93</v>
+        <v>0.99</v>
       </c>
       <c r="U14">
-        <v>0.71</v>
+        <v>0.96</v>
       </c>
       <c r="V14">
         <v>0.15</v>
@@ -16380,19 +16380,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E25">
-        <v>172.09</v>
+        <v>170.95</v>
       </c>
       <c r="F25">
-        <v>-80.6</v>
+        <v>-78.93</v>
       </c>
       <c r="G25">
         <v>378.3</v>
       </c>
       <c r="H25">
-        <v>12.97</v>
+        <v>14.34</v>
       </c>
       <c r="I25">
-        <v>16.4</v>
+        <v>10.2</v>
       </c>
       <c r="J25">
         <v>2.75</v>
@@ -16419,16 +16419,16 @@
         <v>73.7</v>
       </c>
       <c r="R25">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="S25">
         <v>0.67</v>
       </c>
       <c r="T25">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="U25">
-        <v>0.79</v>
+        <v>0.75</v>
       </c>
       <c r="V25">
         <v>0.15</v>
@@ -16454,19 +16454,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E26">
-        <v>157.75</v>
+        <v>156.82</v>
       </c>
       <c r="F26">
-        <v>-78.99</v>
+        <v>-78.93</v>
       </c>
       <c r="G26">
         <v>378.3</v>
       </c>
       <c r="H26">
-        <v>14.29</v>
+        <v>14.36</v>
       </c>
       <c r="I26">
-        <v>14.3</v>
+        <v>10.6</v>
       </c>
       <c r="J26">
         <v>2.75</v>
@@ -16499,7 +16499,7 @@
         <v>0.67</v>
       </c>
       <c r="T26">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="U26">
         <v>0.75</v>
@@ -16528,19 +16528,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E27">
-        <v>143.31</v>
+        <v>142.07</v>
       </c>
       <c r="F27">
-        <v>-78.94</v>
+        <v>-78.93</v>
       </c>
       <c r="G27">
         <v>378.3</v>
       </c>
       <c r="H27">
-        <v>14.18</v>
+        <v>14.31</v>
       </c>
       <c r="I27">
-        <v>14.5</v>
+        <v>9.7</v>
       </c>
       <c r="J27">
         <v>2.75</v>
@@ -16570,13 +16570,13 @@
         <v>0.73</v>
       </c>
       <c r="S27">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="T27">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="U27">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="V27">
         <v>0.15</v>
@@ -16602,19 +16602,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E28">
-        <v>128.93</v>
+        <v>127.95</v>
       </c>
       <c r="F28">
-        <v>-79.36</v>
+        <v>-78.93</v>
       </c>
       <c r="G28">
         <v>378.3</v>
       </c>
       <c r="H28">
-        <v>14.12</v>
+        <v>14.34</v>
       </c>
       <c r="I28">
-        <v>14.4</v>
+        <v>10.2</v>
       </c>
       <c r="J28">
         <v>2.75</v>
@@ -16647,10 +16647,10 @@
         <v>0.67</v>
       </c>
       <c r="T28">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="U28">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="V28">
         <v>0.15</v>
@@ -16676,19 +16676,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E29">
-        <v>114.44</v>
+        <v>113.2</v>
       </c>
       <c r="F29">
-        <v>-78.94</v>
+        <v>-78.93</v>
       </c>
       <c r="G29">
         <v>378.3</v>
       </c>
       <c r="H29">
-        <v>14.17</v>
+        <v>14.29</v>
       </c>
       <c r="I29">
-        <v>14</v>
+        <v>9.2</v>
       </c>
       <c r="J29">
         <v>2.75</v>
@@ -16715,16 +16715,16 @@
         <v>73.7</v>
       </c>
       <c r="R29">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="S29">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="T29">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="U29">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="V29">
         <v>0.15</v>
@@ -16750,34 +16750,34 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E30">
-        <v>371.71</v>
+        <v>369.3</v>
       </c>
       <c r="F30">
-        <v>-73.49</v>
+        <v>-73.82</v>
       </c>
       <c r="G30">
         <v>378.3</v>
       </c>
       <c r="H30">
-        <v>20.76</v>
+        <v>21.3</v>
       </c>
       <c r="I30">
-        <v>14.4</v>
+        <v>8.3</v>
       </c>
       <c r="J30">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="K30">
         <v>0.4</v>
       </c>
       <c r="L30">
-        <v>2.48</v>
+        <v>3.01</v>
       </c>
       <c r="M30">
-        <v>119</v>
+        <v>141</v>
       </c>
       <c r="N30">
-        <v>6.4</v>
+        <v>7.7</v>
       </c>
       <c r="O30">
         <v>4</v>
@@ -16789,16 +16789,16 @@
         <v>87.3</v>
       </c>
       <c r="R30">
-        <v>0.61</v>
+        <v>0.56</v>
       </c>
       <c r="S30">
-        <v>0.92</v>
+        <v>0.81</v>
       </c>
       <c r="T30">
-        <v>0.94</v>
+        <v>0.84</v>
       </c>
       <c r="U30">
-        <v>0.98</v>
+        <v>0.66</v>
       </c>
       <c r="V30">
         <v>0.15</v>
@@ -16898,19 +16898,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E32">
-        <v>337.83</v>
+        <v>346.24</v>
       </c>
       <c r="F32">
-        <v>-69.35</v>
+        <v>-75.68</v>
       </c>
       <c r="G32">
         <v>378.3</v>
       </c>
       <c r="H32">
-        <v>22.08</v>
+        <v>21.45</v>
       </c>
       <c r="I32">
-        <v>2.5</v>
+        <v>26.3</v>
       </c>
       <c r="J32">
         <v>2.75</v>
@@ -16937,16 +16937,16 @@
         <v>87.3</v>
       </c>
       <c r="R32">
-        <v>0.5</v>
+        <v>0.56</v>
       </c>
       <c r="S32">
+        <v>0.81</v>
+      </c>
+      <c r="T32">
         <v>0.83</v>
       </c>
-      <c r="T32">
-        <v>0.87</v>
-      </c>
       <c r="U32">
-        <v>0.74</v>
+        <v>0.65</v>
       </c>
       <c r="V32">
         <v>0.15</v>
@@ -16972,19 +16972,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E33">
-        <v>111.96</v>
+        <v>110.63</v>
       </c>
       <c r="F33">
-        <v>89.82</v>
+        <v>90.49</v>
       </c>
       <c r="G33">
         <v>378.3</v>
       </c>
       <c r="H33">
-        <v>10.67</v>
+        <v>11.52</v>
       </c>
       <c r="I33">
-        <v>355.2</v>
+        <v>348.9</v>
       </c>
       <c r="J33">
         <v>2.5</v>
@@ -17017,10 +17017,10 @@
         <v>0.59</v>
       </c>
       <c r="T33">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="U33">
-        <v>0.95</v>
+        <v>0.89</v>
       </c>
       <c r="V33">
         <v>0.15</v>
@@ -17049,16 +17049,16 @@
         <v>130.63</v>
       </c>
       <c r="F34">
-        <v>93.62</v>
+        <v>90.49</v>
       </c>
       <c r="G34">
         <v>378.3</v>
       </c>
       <c r="H34">
-        <v>11.6</v>
+        <v>13.97</v>
       </c>
       <c r="I34">
-        <v>330.3</v>
+        <v>324</v>
       </c>
       <c r="J34">
         <v>2.5</v>
@@ -17085,16 +17085,16 @@
         <v>59.1</v>
       </c>
       <c r="R34">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="S34">
         <v>0.59</v>
       </c>
       <c r="T34">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="U34">
-        <v>0.74</v>
+        <v>0.65</v>
       </c>
       <c r="V34">
         <v>0.15</v>
@@ -17123,16 +17123,16 @@
         <v>83.63</v>
       </c>
       <c r="F35">
-        <v>87.37</v>
+        <v>90.49</v>
       </c>
       <c r="G35">
         <v>378.3</v>
       </c>
       <c r="H35">
-        <v>8.79</v>
+        <v>11.75</v>
       </c>
       <c r="I35">
-        <v>338.5</v>
+        <v>344.1</v>
       </c>
       <c r="J35">
         <v>2.5</v>
@@ -17165,10 +17165,10 @@
         <v>0.59</v>
       </c>
       <c r="T35">
-        <v>0.94</v>
+        <v>0.89</v>
       </c>
       <c r="U35">
-        <v>0.98</v>
+        <v>0.87</v>
       </c>
       <c r="V35">
         <v>0.15</v>
@@ -17268,19 +17268,19 @@
         <v>DÙNG CHUNG</v>
       </c>
       <c r="E37">
-        <v>115.24</v>
+        <v>121.79</v>
       </c>
       <c r="F37">
-        <v>293.32</v>
+        <v>292.95</v>
       </c>
       <c r="G37">
         <v>378.3</v>
       </c>
       <c r="H37">
-        <v>12.14</v>
+        <v>11.49</v>
       </c>
       <c r="I37">
-        <v>341.8</v>
+        <v>13.8</v>
       </c>
       <c r="J37">
         <v>2.5</v>
@@ -17307,16 +17307,16 @@
         <v>59.1</v>
       </c>
       <c r="R37">
-        <v>0.67</v>
+        <v>0.73</v>
       </c>
       <c r="S37">
-        <v>0.87</v>
+        <v>0.59</v>
       </c>
       <c r="T37">
-        <v>0.94</v>
+        <v>0.86</v>
       </c>
       <c r="U37">
-        <v>0.98</v>
+        <v>0.82</v>
       </c>
       <c r="V37">
         <v>0.15</v>
@@ -17376,7 +17376,7 @@
         <v>Tổng bê tông đế</v>
       </c>
       <c r="B43">
-        <v>93.4</v>
+        <v>92.2</v>
       </c>
       <c r="C43" t="str">
         <v>m³</v>
@@ -17387,7 +17387,7 @@
         <v>Tổng thép bản đế (ước tính)</v>
       </c>
       <c r="B44">
-        <v>4.42</v>
+        <v>4.36</v>
       </c>
       <c r="C44" t="str">
         <v>tấn</v>
@@ -17561,19 +17561,19 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F4">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="G4">
-        <v>28.9</v>
+        <v>29.7</v>
       </c>
       <c r="H4">
         <v>30.1</v>
       </c>
       <c r="I4">
-        <v>14.6</v>
+        <v>15</v>
       </c>
       <c r="J4">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="K4">
         <v>0.33</v>
@@ -17614,16 +17614,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F5">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="G5">
-        <v>36.8</v>
+        <v>36.5</v>
       </c>
       <c r="H5">
         <v>27.6</v>
       </c>
       <c r="I5">
-        <v>16.6</v>
+        <v>16.5</v>
       </c>
       <c r="J5">
         <v>0.25</v>
@@ -17667,19 +17667,19 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F6">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>35.3</v>
+        <v>36.5</v>
       </c>
       <c r="H6">
         <v>38.4</v>
       </c>
       <c r="I6">
-        <v>22.3</v>
+        <v>23</v>
       </c>
       <c r="J6">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="K6">
         <v>0.42</v>
@@ -17688,7 +17688,7 @@
         <v>0.54</v>
       </c>
       <c r="M6">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="N6">
         <v>0.15</v>
@@ -17720,19 +17720,19 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F7">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="G7">
-        <v>35</v>
+        <v>35.6</v>
       </c>
       <c r="H7">
         <v>73.3</v>
       </c>
       <c r="I7">
-        <v>42.2</v>
+        <v>42.8</v>
       </c>
       <c r="J7">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="K7">
         <v>0.72</v>
@@ -17741,7 +17741,7 @@
         <v>0.92</v>
       </c>
       <c r="M7">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="N7">
         <v>0.15</v>
@@ -17826,28 +17826,28 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F9">
-        <v>6.2</v>
+        <v>4.8</v>
       </c>
       <c r="G9">
-        <v>37.4</v>
+        <v>30.5</v>
       </c>
       <c r="H9">
-        <v>45.3</v>
+        <v>45.4</v>
       </c>
       <c r="I9">
-        <v>27.7</v>
+        <v>23.1</v>
       </c>
       <c r="J9">
-        <v>0.42</v>
+        <v>0.35</v>
       </c>
       <c r="K9">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="L9">
-        <v>0.65</v>
+        <v>0.6</v>
       </c>
       <c r="M9">
-        <v>0.33</v>
+        <v>0.22</v>
       </c>
       <c r="N9">
         <v>0.15</v>
@@ -17985,25 +17985,25 @@
         <v>Ø12 a200</v>
       </c>
       <c r="F12">
-        <v>3.8</v>
+        <v>4.8</v>
       </c>
       <c r="G12">
-        <v>25.1</v>
+        <v>30.3</v>
       </c>
       <c r="H12">
         <v>30.8</v>
       </c>
       <c r="I12">
-        <v>13.1</v>
+        <v>15.6</v>
       </c>
       <c r="J12">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="K12">
         <v>0.34</v>
       </c>
       <c r="L12">
-        <v>0.38</v>
+        <v>0.41</v>
       </c>
       <c r="M12">
         <v>0</v>
@@ -18328,7 +18328,7 @@
         <v>30.2</v>
       </c>
       <c r="G8">
-        <v>11.7</v>
+        <v>11.3</v>
       </c>
       <c r="H8" t="str">
         <v>B2-D20</v>
@@ -18340,19 +18340,19 @@
         <v>27.8</v>
       </c>
       <c r="K8">
-        <v>11.07</v>
+        <v>11.3</v>
       </c>
       <c r="L8">
-        <v>-139.37</v>
+        <v>-138.58</v>
       </c>
       <c r="M8">
-        <v>30.03</v>
+        <v>31.21</v>
       </c>
       <c r="N8">
         <v>378.3</v>
       </c>
       <c r="O8">
-        <v>378.87</v>
+        <v>378.71</v>
       </c>
       <c r="P8">
         <v>1.7</v>
@@ -18364,10 +18364,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S8">
-        <v>6.4</v>
+        <v>2.1</v>
       </c>
       <c r="T8">
-        <v>30.8</v>
+        <v>31</v>
       </c>
       <c r="U8">
         <v>2.5</v>
@@ -18391,10 +18391,10 @@
         <v>0.47</v>
       </c>
       <c r="AB8">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="AC8">
-        <v>0.5</v>
+        <v>0.47</v>
       </c>
       <c r="AD8">
         <v>0</v>
@@ -18412,7 +18412,7 @@
         <v>ĐẠT</v>
       </c>
       <c r="AI8" t="str">
-        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 0,6 m: kiểm tra khảo sát / nạo vét trước khi đặt đế</v>
+        <v>Đế dùng chung hai bè: hai tai neo</v>
       </c>
     </row>
     <row r="9">
@@ -18542,7 +18542,7 @@
         <v>27.8</v>
       </c>
       <c r="G10">
-        <v>8.91</v>
+        <v>9.01</v>
       </c>
       <c r="H10" t="str">
         <v>B3-D17</v>
@@ -18554,13 +18554,13 @@
         <v>38.6</v>
       </c>
       <c r="K10">
-        <v>9.44</v>
+        <v>9.02</v>
       </c>
       <c r="L10">
-        <v>-48.11</v>
+        <v>-48.54</v>
       </c>
       <c r="M10">
-        <v>-33.37</v>
+        <v>-35.03</v>
       </c>
       <c r="N10">
         <v>378.3</v>
@@ -18578,10 +18578,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S10">
-        <v>13.3</v>
+        <v>8.5</v>
       </c>
       <c r="T10">
-        <v>40.7</v>
+        <v>41.3</v>
       </c>
       <c r="U10">
         <v>2.5</v>
@@ -18602,16 +18602,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA10">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="AB10">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="AC10">
-        <v>0.69</v>
+        <v>0.67</v>
       </c>
       <c r="AD10">
-        <v>0.43</v>
+        <v>0.38</v>
       </c>
       <c r="AE10">
         <v>0.15</v>
@@ -18620,7 +18620,7 @@
         <v>0.62</v>
       </c>
       <c r="AG10">
-        <v>0.69</v>
+        <v>0.67</v>
       </c>
       <c r="AH10" t="str">
         <v>ĐẠT</v>
@@ -18649,7 +18649,7 @@
         <v>27.8</v>
       </c>
       <c r="G11">
-        <v>13.98</v>
+        <v>14.23</v>
       </c>
       <c r="H11" t="str">
         <v>B3-D13</v>
@@ -18661,19 +18661,19 @@
         <v>38.6</v>
       </c>
       <c r="K11">
-        <v>15.72</v>
+        <v>14.23</v>
       </c>
       <c r="L11">
-        <v>-25.86</v>
+        <v>-28.46</v>
       </c>
       <c r="M11">
-        <v>-15.46</v>
+        <v>-18.93</v>
       </c>
       <c r="N11">
         <v>378.3</v>
       </c>
       <c r="O11">
-        <v>378.54</v>
+        <v>378.5</v>
       </c>
       <c r="P11">
         <v>1.7</v>
@@ -18685,10 +18685,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S11">
-        <v>19.9</v>
+        <v>9.7</v>
       </c>
       <c r="T11">
-        <v>28.6</v>
+        <v>29.8</v>
       </c>
       <c r="U11">
         <v>2.5</v>
@@ -18709,16 +18709,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA11">
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="AB11">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="AC11">
-        <v>0.56</v>
+        <v>0.51</v>
       </c>
       <c r="AD11">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
       <c r="AE11">
         <v>0.15</v>
@@ -18756,7 +18756,7 @@
         <v>38.6</v>
       </c>
       <c r="G12">
-        <v>9.54</v>
+        <v>9.36</v>
       </c>
       <c r="H12" t="str">
         <v>B3A-D23</v>
@@ -18768,13 +18768,13 @@
         <v>73.7</v>
       </c>
       <c r="K12">
-        <v>9.56</v>
+        <v>9.35</v>
       </c>
       <c r="L12">
-        <v>18.01</v>
+        <v>16.6</v>
       </c>
       <c r="M12">
-        <v>-122.77</v>
+        <v>-124.06</v>
       </c>
       <c r="N12">
         <v>378.3</v>
@@ -18792,10 +18792,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S12">
-        <v>32.9</v>
+        <v>27.8</v>
       </c>
       <c r="T12">
-        <v>67.3</v>
+        <v>68.2</v>
       </c>
       <c r="U12">
         <v>3.25</v>
@@ -18816,16 +18816,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA12">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="AB12">
-        <v>0.62</v>
+        <v>0.55</v>
       </c>
       <c r="AC12">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="AD12">
-        <v>0.71</v>
+        <v>0.68</v>
       </c>
       <c r="AE12">
         <v>0.15</v>
@@ -18834,7 +18834,7 @@
         <v>0.62</v>
       </c>
       <c r="AG12">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="AH12" t="str">
         <v>ĐẠT</v>
@@ -18863,7 +18863,7 @@
         <v>38.6</v>
       </c>
       <c r="G13">
-        <v>18.74</v>
+        <v>15.33</v>
       </c>
       <c r="H13" t="str">
         <v>B3A-D21</v>
@@ -18875,19 +18875,19 @@
         <v>73.7</v>
       </c>
       <c r="K13">
-        <v>15.18</v>
+        <v>15.33</v>
       </c>
       <c r="L13">
-        <v>49.15</v>
+        <v>42.39</v>
       </c>
       <c r="M13">
-        <v>-116.18</v>
+        <v>-119.37</v>
       </c>
       <c r="N13">
         <v>378.3</v>
       </c>
       <c r="O13">
-        <v>378.89</v>
+        <v>378.5</v>
       </c>
       <c r="P13">
         <v>1.7</v>
@@ -18899,40 +18899,40 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S13">
-        <v>52.1</v>
+        <v>31.7</v>
       </c>
       <c r="T13">
-        <v>45.2</v>
+        <v>47.5</v>
       </c>
       <c r="U13">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="V13">
         <v>0.4</v>
       </c>
       <c r="W13">
-        <v>45.4</v>
+        <v>37.5</v>
       </c>
       <c r="X13">
-        <v>3.01</v>
+        <v>2.48</v>
       </c>
       <c r="Y13">
-        <v>7.7</v>
+        <v>6.4</v>
       </c>
       <c r="Z13" t="str">
         <v>Ø12 a200</v>
       </c>
       <c r="AA13">
-        <v>0.62</v>
+        <v>0.73</v>
       </c>
       <c r="AB13">
-        <v>0.69</v>
+        <v>0.75</v>
       </c>
       <c r="AC13">
         <v>0.91</v>
       </c>
       <c r="AD13">
-        <v>0.84</v>
+        <v>0.93</v>
       </c>
       <c r="AE13">
         <v>0.15</v>
@@ -18941,13 +18941,13 @@
         <v>0.62</v>
       </c>
       <c r="AG13">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="AH13" t="str">
         <v>ĐẠT</v>
       </c>
       <c r="AI13" t="str">
-        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 0,6 m: kiểm tra khảo sát / nạo vét trước khi đặt đế; Đế lớn hơn đế mẫu</v>
+        <v>Đế dùng chung hai bè: hai tai neo</v>
       </c>
     </row>
     <row r="14">
@@ -18970,7 +18970,7 @@
         <v>38.6</v>
       </c>
       <c r="G14">
-        <v>14.3</v>
+        <v>12.34</v>
       </c>
       <c r="H14" t="str">
         <v>B3A-D22</v>
@@ -18982,13 +18982,13 @@
         <v>73.7</v>
       </c>
       <c r="K14">
-        <v>11.97</v>
+        <v>12.34</v>
       </c>
       <c r="L14">
-        <v>33.69</v>
+        <v>29.5</v>
       </c>
       <c r="M14">
-        <v>-119.71</v>
+        <v>-121.71</v>
       </c>
       <c r="N14">
         <v>378.3</v>
@@ -19006,40 +19006,40 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S14">
-        <v>43.1</v>
+        <v>30.3</v>
       </c>
       <c r="T14">
-        <v>55.1</v>
+        <v>56.3</v>
       </c>
       <c r="U14">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="V14">
         <v>0.4</v>
       </c>
       <c r="W14">
-        <v>54</v>
+        <v>45.4</v>
       </c>
       <c r="X14">
-        <v>3.58</v>
+        <v>3.01</v>
       </c>
       <c r="Y14">
-        <v>9.2</v>
+        <v>7.7</v>
       </c>
       <c r="Z14" t="str">
         <v>Ø12 a200</v>
       </c>
       <c r="AA14">
-        <v>0.69</v>
+        <v>0.78</v>
       </c>
       <c r="AB14">
-        <v>0.83</v>
+        <v>0.67</v>
       </c>
       <c r="AC14">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="AD14">
-        <v>0.74</v>
+        <v>0.92</v>
       </c>
       <c r="AE14">
         <v>0.15</v>
@@ -19048,7 +19048,7 @@
         <v>0.62</v>
       </c>
       <c r="AG14">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="AH14" t="str">
         <v>ĐẠT</v>
@@ -19077,7 +19077,7 @@
         <v>38.6</v>
       </c>
       <c r="G15">
-        <v>9.76</v>
+        <v>9.6</v>
       </c>
       <c r="H15" t="str">
         <v>B3A-D24</v>
@@ -19089,13 +19089,13 @@
         <v>73.7</v>
       </c>
       <c r="K15">
-        <v>12.73</v>
+        <v>9.59</v>
       </c>
       <c r="L15">
-        <v>0.59</v>
+        <v>5.97</v>
       </c>
       <c r="M15">
-        <v>-131.46</v>
+        <v>-128.68</v>
       </c>
       <c r="N15">
         <v>378.3</v>
@@ -19113,40 +19113,40 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S15">
-        <v>57.5</v>
+        <v>28.1</v>
       </c>
       <c r="T15">
-        <v>58.9</v>
+        <v>67.1</v>
       </c>
       <c r="U15">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="V15">
         <v>0.4</v>
       </c>
       <c r="W15">
-        <v>63.4</v>
+        <v>54</v>
       </c>
       <c r="X15">
-        <v>4.21</v>
+        <v>3.58</v>
       </c>
       <c r="Y15">
-        <v>10.8</v>
+        <v>9.2</v>
       </c>
       <c r="Z15" t="str">
         <v>Ø12 a200</v>
       </c>
       <c r="AA15">
-        <v>0.66</v>
+        <v>0.84</v>
       </c>
       <c r="AB15">
-        <v>0.58</v>
+        <v>0.61</v>
       </c>
       <c r="AC15">
-        <v>0.93</v>
+        <v>0.99</v>
       </c>
       <c r="AD15">
-        <v>0.71</v>
+        <v>0.96</v>
       </c>
       <c r="AE15">
         <v>0.15</v>
@@ -19155,7 +19155,7 @@
         <v>0.62</v>
       </c>
       <c r="AG15">
-        <v>0.93</v>
+        <v>0.99</v>
       </c>
       <c r="AH15" t="str">
         <v>ĐẠT</v>
@@ -20254,7 +20254,7 @@
         <v>73.7</v>
       </c>
       <c r="G26">
-        <v>12.97</v>
+        <v>14.34</v>
       </c>
       <c r="H26" t="str">
         <v>B7-D23</v>
@@ -20266,13 +20266,13 @@
         <v>45.6</v>
       </c>
       <c r="K26">
-        <v>15.85</v>
+        <v>14.34</v>
       </c>
       <c r="L26">
-        <v>172.09</v>
+        <v>170.95</v>
       </c>
       <c r="M26">
-        <v>-80.6</v>
+        <v>-78.93</v>
       </c>
       <c r="N26">
         <v>378.3</v>
@@ -20290,10 +20290,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S26">
-        <v>25.2</v>
+        <v>25.1</v>
       </c>
       <c r="T26">
-        <v>54.3</v>
+        <v>53.2</v>
       </c>
       <c r="U26">
         <v>2.75</v>
@@ -20314,16 +20314,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA26">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="AB26">
         <v>0.67</v>
       </c>
       <c r="AC26">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="AD26">
-        <v>0.79</v>
+        <v>0.75</v>
       </c>
       <c r="AE26">
         <v>0.15</v>
@@ -20332,7 +20332,7 @@
         <v>0.62</v>
       </c>
       <c r="AG26">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="AH26" t="str">
         <v>ĐẠT</v>
@@ -20361,7 +20361,7 @@
         <v>73.7</v>
       </c>
       <c r="G27">
-        <v>14.5</v>
+        <v>14.36</v>
       </c>
       <c r="H27" t="str">
         <v>B7-D32</v>
@@ -20373,13 +20373,13 @@
         <v>45.6</v>
       </c>
       <c r="K27">
-        <v>14.29</v>
+        <v>14.37</v>
       </c>
       <c r="L27">
-        <v>157.75</v>
+        <v>156.82</v>
       </c>
       <c r="M27">
-        <v>-78.99</v>
+        <v>-78.93</v>
       </c>
       <c r="N27">
         <v>378.3</v>
@@ -20397,10 +20397,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S27">
-        <v>26.2</v>
+        <v>25.1</v>
       </c>
       <c r="T27">
-        <v>53</v>
+        <v>53.1</v>
       </c>
       <c r="U27">
         <v>2.75</v>
@@ -20427,7 +20427,7 @@
         <v>0.67</v>
       </c>
       <c r="AC27">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AD27">
         <v>0.75</v>
@@ -20439,7 +20439,7 @@
         <v>0.62</v>
       </c>
       <c r="AG27">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AH27" t="str">
         <v>ĐẠT</v>
@@ -20468,7 +20468,7 @@
         <v>73.7</v>
       </c>
       <c r="G28">
-        <v>14.56</v>
+        <v>14.31</v>
       </c>
       <c r="H28" t="str">
         <v>B7-D19</v>
@@ -20480,13 +20480,13 @@
         <v>45.6</v>
       </c>
       <c r="K28">
-        <v>14.18</v>
+        <v>14.32</v>
       </c>
       <c r="L28">
-        <v>143.31</v>
+        <v>142.07</v>
       </c>
       <c r="M28">
-        <v>-78.94</v>
+        <v>-78.93</v>
       </c>
       <c r="N28">
         <v>378.3</v>
@@ -20504,10 +20504,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S28">
-        <v>26.9</v>
+        <v>25.1</v>
       </c>
       <c r="T28">
-        <v>53</v>
+        <v>53.3</v>
       </c>
       <c r="U28">
         <v>2.75</v>
@@ -20531,13 +20531,13 @@
         <v>0.73</v>
       </c>
       <c r="AB28">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="AC28">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AD28">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="AE28">
         <v>0.15</v>
@@ -20546,7 +20546,7 @@
         <v>0.62</v>
       </c>
       <c r="AG28">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AH28" t="str">
         <v>ĐẠT</v>
@@ -20575,7 +20575,7 @@
         <v>73.7</v>
       </c>
       <c r="G29">
-        <v>14.12</v>
+        <v>14.34</v>
       </c>
       <c r="H29" t="str">
         <v>B7-D31</v>
@@ -20587,13 +20587,13 @@
         <v>45.6</v>
       </c>
       <c r="K29">
-        <v>14.63</v>
+        <v>14.34</v>
       </c>
       <c r="L29">
-        <v>128.93</v>
+        <v>127.95</v>
       </c>
       <c r="M29">
-        <v>-79.36</v>
+        <v>-78.93</v>
       </c>
       <c r="N29">
         <v>378.3</v>
@@ -20611,10 +20611,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S29">
-        <v>25.9</v>
+        <v>25.1</v>
       </c>
       <c r="T29">
-        <v>53.3</v>
+        <v>53.2</v>
       </c>
       <c r="U29">
         <v>2.75</v>
@@ -20641,10 +20641,10 @@
         <v>0.67</v>
       </c>
       <c r="AC29">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AD29">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="AE29">
         <v>0.15</v>
@@ -20653,7 +20653,7 @@
         <v>0.62</v>
       </c>
       <c r="AG29">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AH29" t="str">
         <v>ĐẠT</v>
@@ -20682,7 +20682,7 @@
         <v>73.7</v>
       </c>
       <c r="G30">
-        <v>14.53</v>
+        <v>14.29</v>
       </c>
       <c r="H30" t="str">
         <v>B7-D22</v>
@@ -20694,13 +20694,13 @@
         <v>45.6</v>
       </c>
       <c r="K30">
-        <v>14.17</v>
+        <v>14.3</v>
       </c>
       <c r="L30">
-        <v>114.44</v>
+        <v>113.2</v>
       </c>
       <c r="M30">
-        <v>-78.94</v>
+        <v>-78.93</v>
       </c>
       <c r="N30">
         <v>378.3</v>
@@ -20718,10 +20718,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S30">
-        <v>26.9</v>
+        <v>25.1</v>
       </c>
       <c r="T30">
-        <v>53.1</v>
+        <v>53.3</v>
       </c>
       <c r="U30">
         <v>2.75</v>
@@ -20742,16 +20742,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA30">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="AB30">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="AC30">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AD30">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="AE30">
         <v>0.15</v>
@@ -20760,7 +20760,7 @@
         <v>0.62</v>
       </c>
       <c r="AG30">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="AH30" t="str">
         <v>ĐẠT</v>
@@ -20789,7 +20789,7 @@
         <v>87.3</v>
       </c>
       <c r="G31">
-        <v>22.11</v>
+        <v>21.31</v>
       </c>
       <c r="H31" t="str">
         <v>B6-D27</v>
@@ -20801,19 +20801,19 @@
         <v>40.8</v>
       </c>
       <c r="K31">
-        <v>20.76</v>
+        <v>21.3</v>
       </c>
       <c r="L31">
-        <v>371.71</v>
+        <v>369.3</v>
       </c>
       <c r="M31">
-        <v>-73.49</v>
+        <v>-73.82</v>
       </c>
       <c r="N31">
         <v>378.3</v>
       </c>
       <c r="O31">
-        <v>381.41</v>
+        <v>381.37</v>
       </c>
       <c r="P31">
         <v>1.7</v>
@@ -20825,40 +20825,40 @@
         <v>B5A-D13 căng, B6-D27 chùng (MN cao)</v>
       </c>
       <c r="S31">
-        <v>78.5</v>
+        <v>78.1</v>
       </c>
       <c r="T31">
-        <v>28.5</v>
+        <v>29.4</v>
       </c>
       <c r="U31">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="V31">
         <v>0.4</v>
       </c>
       <c r="W31">
-        <v>37.5</v>
+        <v>45.4</v>
       </c>
       <c r="X31">
-        <v>2.48</v>
+        <v>3.01</v>
       </c>
       <c r="Y31">
-        <v>6.4</v>
+        <v>7.7</v>
       </c>
       <c r="Z31" t="str">
         <v>Ø12 a200</v>
       </c>
       <c r="AA31">
-        <v>0.61</v>
+        <v>0.56</v>
       </c>
       <c r="AB31">
-        <v>0.92</v>
+        <v>0.81</v>
       </c>
       <c r="AC31">
-        <v>0.94</v>
+        <v>0.84</v>
       </c>
       <c r="AD31">
-        <v>0.98</v>
+        <v>0.66</v>
       </c>
       <c r="AE31">
         <v>0.15</v>
@@ -20867,13 +20867,13 @@
         <v>0.62</v>
       </c>
       <c r="AG31">
-        <v>0.98</v>
+        <v>0.84</v>
       </c>
       <c r="AH31" t="str">
         <v>ĐẠT</v>
       </c>
       <c r="AI31" t="str">
-        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 3,1 m: kiểm tra khảo sát / nạo vét trước khi đặt đế</v>
+        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 3,1 m: kiểm tra khảo sát / nạo vét trước khi đặt đế; Đế lớn hơn đế mẫu</v>
       </c>
     </row>
     <row r="32">
@@ -21003,7 +21003,7 @@
         <v>87.3</v>
       </c>
       <c r="G33">
-        <v>25.58</v>
+        <v>21.46</v>
       </c>
       <c r="H33" t="str">
         <v>B6-D17</v>
@@ -21015,19 +21015,19 @@
         <v>40.8</v>
       </c>
       <c r="K33">
-        <v>22.08</v>
+        <v>21.45</v>
       </c>
       <c r="L33">
-        <v>337.83</v>
+        <v>346.24</v>
       </c>
       <c r="M33">
-        <v>-69.35</v>
+        <v>-75.68</v>
       </c>
       <c r="N33">
         <v>378.3</v>
       </c>
       <c r="O33">
-        <v>381.18</v>
+        <v>381.05</v>
       </c>
       <c r="P33">
         <v>1.7</v>
@@ -21036,13 +21036,13 @@
         <v>7.7</v>
       </c>
       <c r="R33" t="str">
-        <v>cả hai dây căng (MN cao)</v>
+        <v>B5A-D15 căng, B6-D17 chùng (MN cao)</v>
       </c>
       <c r="S33">
-        <v>67.4</v>
+        <v>78.1</v>
       </c>
       <c r="T33">
-        <v>36.1</v>
+        <v>29.2</v>
       </c>
       <c r="U33">
         <v>2.75</v>
@@ -21063,16 +21063,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA33">
-        <v>0.5</v>
+        <v>0.56</v>
       </c>
       <c r="AB33">
+        <v>0.81</v>
+      </c>
+      <c r="AC33">
         <v>0.83</v>
       </c>
-      <c r="AC33">
-        <v>0.87</v>
-      </c>
       <c r="AD33">
-        <v>0.74</v>
+        <v>0.65</v>
       </c>
       <c r="AE33">
         <v>0.15</v>
@@ -21081,13 +21081,13 @@
         <v>0.62</v>
       </c>
       <c r="AG33">
-        <v>0.87</v>
+        <v>0.83</v>
       </c>
       <c r="AH33" t="str">
         <v>ĐẠT</v>
       </c>
       <c r="AI33" t="str">
-        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 2,9 m: kiểm tra khảo sát / nạo vét trước khi đặt đế; Đế lớn hơn đế mẫu</v>
+        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 2,8 m: kiểm tra khảo sát / nạo vét trước khi đặt đế; Đế lớn hơn đế mẫu</v>
       </c>
     </row>
     <row r="34">
@@ -21110,7 +21110,7 @@
         <v>45.6</v>
       </c>
       <c r="G34">
-        <v>10.67</v>
+        <v>11.52</v>
       </c>
       <c r="H34" t="str">
         <v>B8-D31</v>
@@ -21122,13 +21122,13 @@
         <v>59.1</v>
       </c>
       <c r="K34">
-        <v>12.49</v>
+        <v>11.52</v>
       </c>
       <c r="L34">
-        <v>111.96</v>
+        <v>110.63</v>
       </c>
       <c r="M34">
-        <v>89.82</v>
+        <v>90.49</v>
       </c>
       <c r="N34">
         <v>378.3</v>
@@ -21146,10 +21146,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S34">
-        <v>16.2</v>
+        <v>11.5</v>
       </c>
       <c r="T34">
-        <v>54.7</v>
+        <v>55.2</v>
       </c>
       <c r="U34">
         <v>2.5</v>
@@ -21176,10 +21176,10 @@
         <v>0.59</v>
       </c>
       <c r="AC34">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="AD34">
-        <v>0.95</v>
+        <v>0.89</v>
       </c>
       <c r="AE34">
         <v>0.15</v>
@@ -21188,7 +21188,7 @@
         <v>0.62</v>
       </c>
       <c r="AG34">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="AH34" t="str">
         <v>ĐẠT</v>
@@ -21217,7 +21217,7 @@
         <v>45.6</v>
       </c>
       <c r="G35">
-        <v>16.61</v>
+        <v>13.97</v>
       </c>
       <c r="H35" t="str">
         <v>B8-D32</v>
@@ -21229,13 +21229,13 @@
         <v>59.1</v>
       </c>
       <c r="K35">
-        <v>11.6</v>
+        <v>13.98</v>
       </c>
       <c r="L35">
         <v>130.63</v>
       </c>
       <c r="M35">
-        <v>93.62</v>
+        <v>90.49</v>
       </c>
       <c r="N35">
         <v>378.3</v>
@@ -21253,10 +21253,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S35">
-        <v>15</v>
+        <v>12.1</v>
       </c>
       <c r="T35">
-        <v>49</v>
+        <v>47.7</v>
       </c>
       <c r="U35">
         <v>2.5</v>
@@ -21277,16 +21277,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA35">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="AB35">
         <v>0.59</v>
       </c>
       <c r="AC35">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="AD35">
-        <v>0.74</v>
+        <v>0.65</v>
       </c>
       <c r="AE35">
         <v>0.15</v>
@@ -21295,7 +21295,7 @@
         <v>0.62</v>
       </c>
       <c r="AG35">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="AH35" t="str">
         <v>ĐẠT</v>
@@ -21324,7 +21324,7 @@
         <v>45.6</v>
       </c>
       <c r="G36">
-        <v>8.79</v>
+        <v>11.75</v>
       </c>
       <c r="H36" t="str">
         <v>B8-D29</v>
@@ -21336,13 +21336,13 @@
         <v>59.1</v>
       </c>
       <c r="K36">
-        <v>14.78</v>
+        <v>11.75</v>
       </c>
       <c r="L36">
         <v>83.63</v>
       </c>
       <c r="M36">
-        <v>87.37</v>
+        <v>90.49</v>
       </c>
       <c r="N36">
         <v>378.3</v>
@@ -21360,10 +21360,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S36">
-        <v>19.1</v>
+        <v>11.6</v>
       </c>
       <c r="T36">
-        <v>54.5</v>
+        <v>54.4</v>
       </c>
       <c r="U36">
         <v>2.5</v>
@@ -21390,10 +21390,10 @@
         <v>0.59</v>
       </c>
       <c r="AC36">
-        <v>0.94</v>
+        <v>0.89</v>
       </c>
       <c r="AD36">
-        <v>0.98</v>
+        <v>0.87</v>
       </c>
       <c r="AE36">
         <v>0.15</v>
@@ -21402,7 +21402,7 @@
         <v>0.62</v>
       </c>
       <c r="AG36">
-        <v>0.98</v>
+        <v>0.89</v>
       </c>
       <c r="AH36" t="str">
         <v>ĐẠT</v>
@@ -21538,7 +21538,7 @@
         <v>59.1</v>
       </c>
       <c r="G38">
-        <v>12.14</v>
+        <v>11.49</v>
       </c>
       <c r="H38" t="str">
         <v>B9-D16</v>
@@ -21550,19 +21550,19 @@
         <v>30.9</v>
       </c>
       <c r="K38">
-        <v>14.24</v>
+        <v>11.49</v>
       </c>
       <c r="L38">
-        <v>115.24</v>
+        <v>121.79</v>
       </c>
       <c r="M38">
-        <v>293.32</v>
+        <v>292.95</v>
       </c>
       <c r="N38">
         <v>378.3</v>
       </c>
       <c r="O38">
-        <v>380.69</v>
+        <v>380.8</v>
       </c>
       <c r="P38">
         <v>1.7</v>
@@ -21574,10 +21574,10 @@
         <v>cả hai dây căng (MN cao)</v>
       </c>
       <c r="S38">
-        <v>43.6</v>
+        <v>24</v>
       </c>
       <c r="T38">
-        <v>43.9</v>
+        <v>47.6</v>
       </c>
       <c r="U38">
         <v>2.5</v>
@@ -21598,16 +21598,16 @@
         <v>Ø12 a200</v>
       </c>
       <c r="AA38">
-        <v>0.67</v>
+        <v>0.73</v>
       </c>
       <c r="AB38">
-        <v>0.87</v>
+        <v>0.59</v>
       </c>
       <c r="AC38">
-        <v>0.94</v>
+        <v>0.86</v>
       </c>
       <c r="AD38">
-        <v>0.98</v>
+        <v>0.82</v>
       </c>
       <c r="AE38">
         <v>0.15</v>
@@ -21616,13 +21616,13 @@
         <v>0.62</v>
       </c>
       <c r="AG38">
-        <v>0.98</v>
+        <v>0.86</v>
       </c>
       <c r="AH38" t="str">
         <v>ĐẠT</v>
       </c>
       <c r="AI38" t="str">
-        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 2,4 m: kiểm tra khảo sát / nạo vét trước khi đặt đế</v>
+        <v>Đế dùng chung hai bè: hai tai neo; Địa hình IFC tại điểm này cao hơn đáy thiết kế 2,5 m: kiểm tra khảo sát / nạo vét trước khi đặt đế</v>
       </c>
     </row>
     <row r="39">
@@ -21684,7 +21684,7 @@
         <v>Bê tông đế</v>
       </c>
       <c r="B45">
-        <v>93.4</v>
+        <v>92.2</v>
       </c>
       <c r="C45" t="str">
         <v>m³</v>
@@ -21717,7 +21717,7 @@
         <v>Số đế cạnh B = 2,75 m</v>
       </c>
       <c r="B48">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C48" t="str">
         <v>đế</v>
@@ -21739,7 +21739,7 @@
         <v>Số đế cạnh B = 3,25 m</v>
       </c>
       <c r="B50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="str">
         <v>đế</v>
@@ -21750,7 +21750,7 @@
         <v>Số đế mà địa hình IFC cao hơn đáy thiết kế trên 0,5 m (cần kiểm tra khảo sát / nạo vét)</v>
       </c>
       <c r="B51">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C51" t="str">
         <v>đế</v>
@@ -25490,19 +25490,19 @@
         <v>Chuyển từ neo đáy</v>
       </c>
       <c r="F50">
-        <v>-41.3</v>
+        <v>-35.8</v>
       </c>
       <c r="G50">
-        <v>-149.57</v>
+        <v>-179.26</v>
       </c>
       <c r="H50">
-        <v>384.08</v>
+        <v>385.08</v>
       </c>
       <c r="I50">
-        <v>37.5</v>
+        <v>58</v>
       </c>
       <c r="J50">
-        <v>232</v>
+        <v>204.5</v>
       </c>
       <c r="K50">
         <v>1</v>
@@ -25538,13 +25538,13 @@
         <v>H-8 Cao độ chốt cáp so với yêu cầu thiết kế cọc</v>
       </c>
       <c r="V50">
-        <v>-5.8</v>
+        <v>-4.8</v>
       </c>
       <c r="W50">
-        <v>3.3</v>
+        <v>1.2</v>
       </c>
       <c r="X50" t="str">
-        <v>CÓ</v>
+        <v>không</v>
       </c>
       <c r="Y50" t="str">
         <v>CÓ</v>
@@ -25553,7 +25553,7 @@
         <v>ĐẠT</v>
       </c>
       <c r="AA50" t="str">
-        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ); Mặt đất tại cọc thấp hơn MNDB: thi công mùa nước thấp, có ống vách; Đầu cọc ngập khi hồ ở MNLKT: bản mã, tai neo cần chống gỉ</v>
+        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ); Đầu cọc ngập khi hồ ở MNLKT: bản mã, tai neo cần chống gỉ</v>
       </c>
     </row>
     <row r="51">
@@ -31217,19 +31217,19 @@
         <v>Chuyển từ neo đáy</v>
       </c>
       <c r="F119">
-        <v>419.48</v>
+        <v>423.01</v>
       </c>
       <c r="G119">
-        <v>-154.12</v>
+        <v>-168.16</v>
       </c>
       <c r="H119">
-        <v>384.2</v>
+        <v>388.57</v>
       </c>
       <c r="I119">
-        <v>49.52</v>
+        <v>58.5</v>
       </c>
       <c r="J119">
-        <v>107.9</v>
+        <v>120</v>
       </c>
       <c r="K119">
         <v>1</v>
@@ -31265,22 +31265,22 @@
         <v>H-8 Cao độ chốt cáp so với yêu cầu thiết kế cọc</v>
       </c>
       <c r="V119">
-        <v>-4.6</v>
+        <v>-8.1</v>
       </c>
       <c r="W119">
-        <v>2.4</v>
+        <v>-2.3</v>
       </c>
       <c r="X119" t="str">
-        <v>CÓ</v>
+        <v>không</v>
       </c>
       <c r="Y119" t="str">
-        <v>CÓ</v>
+        <v>không</v>
       </c>
       <c r="Z119" t="str">
         <v>ĐẠT</v>
       </c>
       <c r="AA119" t="str">
-        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ); Mặt đất tại cọc thấp hơn MNDB: thi công mùa nước thấp, có ống vách; Đầu cọc ngập khi hồ ở MNLKT: bản mã, tai neo cần chống gỉ</v>
+        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ)</v>
       </c>
     </row>
     <row r="120">
@@ -31300,19 +31300,19 @@
         <v>Chuyển từ neo đáy</v>
       </c>
       <c r="F120">
-        <v>420.28</v>
+        <v>418.19</v>
       </c>
       <c r="G120">
-        <v>-149.28</v>
+        <v>-162.96</v>
       </c>
       <c r="H120">
-        <v>384.75</v>
+        <v>384</v>
       </c>
       <c r="I120">
-        <v>35</v>
+        <v>39.5</v>
       </c>
       <c r="J120">
-        <v>107.2</v>
+        <v>127.5</v>
       </c>
       <c r="K120">
         <v>1</v>
@@ -31348,13 +31348,13 @@
         <v>H-8 Cao độ chốt cáp so với yêu cầu thiết kế cọc</v>
       </c>
       <c r="V120">
-        <v>-7.3</v>
+        <v>-5.4</v>
       </c>
       <c r="W120">
-        <v>2.5</v>
+        <v>3.3</v>
       </c>
       <c r="X120" t="str">
-        <v>không</v>
+        <v>CÓ</v>
       </c>
       <c r="Y120" t="str">
         <v>CÓ</v>
@@ -31363,7 +31363,7 @@
         <v>ĐẠT</v>
       </c>
       <c r="AA120" t="str">
-        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ); Đầu cọc ngập khi hồ ở MNLKT: bản mã, tai neo cần chống gỉ</v>
+        <v>Chuyển từ neo đáy sang cọc khoan nhồi (vị trí ven bờ); Mặt đất tại cọc thấp hơn MNDB: thi công mùa nước thấp, có ống vách; Đầu cọc ngập khi hồ ở MNLKT: bản mã, tai neo cần chống gỉ</v>
       </c>
     </row>
     <row r="121">
@@ -35616,19 +35616,19 @@
         <v>Chuyển từ neo đáy</v>
       </c>
       <c r="F172">
-        <v>76.46</v>
+        <v>81.73</v>
       </c>
       <c r="G172">
-        <v>-76.01</v>
+        <v>-97.29</v>
       </c>
       <c r="H172">
-        <v>384.07</v>
+        <v>384.1</v>
       </c>
       <c r="I172">
-        <v>26.5</v>
+        <v>37.5</v>
       </c>
       <c r="J172">
-        <v>245</v>
+        <v>210</v>
       </c>
       <c r="K172">
         <v>1</v>
@@ -35664,10 +35664,10 @@
         <v>H-8 Cao độ chốt cáp so với yêu cầu thiết kế cọc</v>
       </c>
       <c r="V172">
-        <v>-8.2</v>
+        <v>-5.9</v>
       </c>
       <c r="W172">
-        <v>4.7</v>
+        <v>3.3</v>
       </c>
       <c r="X172" t="str">
         <v>CÓ</v>
@@ -37940,19 +37940,19 @@
         <v>Chuyển từ neo đáy</v>
       </c>
       <c r="F200">
-        <v>41.03</v>
+        <v>47.33</v>
       </c>
       <c r="G200">
-        <v>92.56</v>
+        <v>71.85</v>
       </c>
       <c r="H200">
-        <v>384.03</v>
+        <v>384.01</v>
       </c>
       <c r="I200">
-        <v>27</v>
+        <v>35.5</v>
       </c>
       <c r="J200">
-        <v>250</v>
+        <v>212.5</v>
       </c>
       <c r="K200">
         <v>1</v>
@@ -37988,10 +37988,10 @@
         <v>H-8 Cao độ chốt cáp so với yêu cầu thiết kế cọc</v>
       </c>
       <c r="V200">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="W200">
-        <v>4.7</v>
+        <v>3.6</v>
       </c>
       <c r="X200" t="str">
         <v>CÓ</v>
@@ -41136,7 +41136,7 @@
         <v>Dây neo bờ dài nhất</v>
       </c>
       <c r="B244">
-        <v>58.4</v>
+        <v>58.5</v>
       </c>
       <c r="C244" t="str">
         <v>m</v>
@@ -41147,7 +41147,7 @@
         <v>Số điểm có mặt đất tại cọc thấp hơn MNDB</v>
       </c>
       <c r="B245">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C245" t="str">
         <v>điểm</v>
@@ -41158,7 +41158,7 @@
         <v>Số điểm có đầu cọc ngập khi hồ ở MNLKT</v>
       </c>
       <c r="B246">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C246" t="str">
         <v>điểm</v>

</xml_diff>